<commit_message>
feat(ai-agent): complete Day 5 SSE streaming and Day 6 pgvector setup
- Day 5: Expose real-time SSE streaming endpoints (/api/v1/agent/stream, /api/agent/stream) powered by Gemini 3.8 Flash live token streaming with PostgreSQL grounding and tenant isolation.
- Day 6: Enable pgvector extension, 04_pgvector.sql migration, recipe_embeddings vector table (768-dim), and cosine similarity functions.
- Update docker-compose.yml to pgvector/pgvector:pg16 and add SQLAlchemy RecipeEmbedding model.
- Add test suites: test_stream.py (npm run test:stream) and verify-pgvector.ts (npm run test:vector).
- Sync sprint roadmap in todo.md and KitchenPluss AI Integration Plan.xlsx (6/20 tasks completed, 30%).
</commit_message>
<xml_diff>
--- a/docs/KitchenPluss AI Integration Plan.xlsx
+++ b/docs/KitchenPluss AI Integration Plan.xlsx
@@ -1242,7 +1242,7 @@
       </c>
       <c r="F11" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="F12" s="28" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
     </row>

</xml_diff>